<commit_message>
fix: add oasis to xlsx ov report
</commit_message>
<xml_diff>
--- a/resources/excel_formats/Bonos_cartera.xlsx
+++ b/resources/excel_formats/Bonos_cartera.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jorge\Google Drive\Django\Andina_stable\resources\excel_formats\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jorge\Mi unidad\Django\Andina_stable\resources\excel_formats\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84C92527-BC0F-40B0-86D0-86402344A5C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44422826-0462-426A-8E97-CE5142401202}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="604" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="604" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Override" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,8 @@
     <sheet name="Vegas de Venecia" sheetId="6" r:id="rId6"/>
     <sheet name="Carmelo Reservado" sheetId="8" r:id="rId7"/>
     <sheet name="Fractal" sheetId="7" r:id="rId8"/>
-    <sheet name="Casas de Verano" sheetId="9" r:id="rId9"/>
+    <sheet name="Oasis" sheetId="10" r:id="rId9"/>
+    <sheet name="Casas de Verano" sheetId="9" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="38">
   <si>
     <t>Gestor</t>
   </si>
@@ -92,15 +93,6 @@
   </si>
   <si>
     <t>Carmelo Reservado</t>
-  </si>
-  <si>
-    <t>SUBTOTAL NELSON SUAREZ CARTERA CCIAL</t>
-  </si>
-  <si>
-    <t>SUBTOTAL NELSON SUAREZ CARTERA ADMIN</t>
-  </si>
-  <si>
-    <t>SUBTOTAL NELSON SUAREZ JEFE CARTERA</t>
   </si>
   <si>
     <t>Cumplimiento (Minimo)</t>
@@ -161,6 +153,9 @@
   </si>
   <si>
     <t>TOTAL NELSON SUAREZ</t>
+  </si>
+  <si>
+    <t>Dina Ortega</t>
   </si>
 </sst>
 </file>
@@ -243,7 +238,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -290,6 +285,19 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -306,7 +314,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -327,7 +335,6 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -343,16 +350,20 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="7" applyFont="1"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="13">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
@@ -679,7 +690,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M24"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="19.21875" customWidth="1"/>
@@ -720,8 +731,8 @@
       <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
@@ -751,14 +762,14 @@
         <v>0</v>
       </c>
       <c r="H2" s="9">
-        <v>1.5E-3</v>
+        <v>2E-3</v>
       </c>
       <c r="I2" s="6">
         <f>+G2*H2</f>
         <v>0</v>
       </c>
       <c r="L2" s="4"/>
-      <c r="M2" s="12"/>
+      <c r="M2" s="11"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
@@ -788,32 +799,32 @@
         <v>0</v>
       </c>
       <c r="H3" s="9">
-        <v>1.5E-3</v>
+        <v>2E-3</v>
       </c>
       <c r="I3" s="6">
         <f>+G3*H3</f>
         <v>0</v>
       </c>
       <c r="L3" s="4"/>
-      <c r="M3" s="12"/>
+      <c r="M3" s="11"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
-      <c r="G4" s="24"/>
-      <c r="H4" s="25"/>
-      <c r="I4" s="19">
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="18">
         <f>SUM(I2:I3)</f>
         <v>0</v>
       </c>
       <c r="L4" s="4"/>
-      <c r="M4" s="12"/>
+      <c r="M4" s="11"/>
     </row>
     <row r="5" spans="1:13" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -844,21 +855,21 @@
         <v>8</v>
       </c>
       <c r="L5" s="4"/>
-      <c r="M5" s="12"/>
+      <c r="M5" s="11"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C6" s="6">
-        <f>+SUMIFS('Tesoro Escondido'!L:L,'Tesoro Escondido'!P:P,Override!A6,'Tesoro Escondido'!F:F,"Comercial")</f>
+        <f>+SUMIFS('Tesoro Escondido'!L:L,'Tesoro Escondido'!P:P,Override!A6)</f>
         <v>0</v>
       </c>
       <c r="D6" s="6">
-        <f>+SUMIFS('Tesoro Escondido'!M:M,'Tesoro Escondido'!P:P,Override!A6,'Tesoro Escondido'!F:F,"Comercial")</f>
+        <f>+SUMIFS('Tesoro Escondido'!M:M,'Tesoro Escondido'!P:P,Override!A6)</f>
         <v>0</v>
       </c>
       <c r="E6" s="7" t="e">
@@ -874,14 +885,14 @@
         <v>0</v>
       </c>
       <c r="H6" s="9">
-        <v>1.5E-3</v>
+        <v>2E-3</v>
       </c>
       <c r="I6" s="6">
         <f>+G6*H6</f>
         <v>0</v>
       </c>
       <c r="L6" s="4"/>
-      <c r="M6" s="12"/>
+      <c r="M6" s="11"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
@@ -891,11 +902,11 @@
         <v>15</v>
       </c>
       <c r="C7" s="6">
-        <f>+SUMIFS('Vegas de Venecia'!L:L,'Vegas de Venecia'!P:P,Override!A7,'Vegas de Venecia'!F:F,"Comercial")</f>
+        <f>+SUMIFS('Vegas de Venecia'!L:L,'Vegas de Venecia'!P:P,Override!A7)</f>
         <v>0</v>
       </c>
       <c r="D7" s="6">
-        <f>+SUMIFS('Vegas de Venecia'!M:M,'Vegas de Venecia'!P:P,Override!A7,'Vegas de Venecia'!F:F,"Comercial")</f>
+        <f>+SUMIFS('Vegas de Venecia'!M:M,'Vegas de Venecia'!P:P,Override!A7)</f>
         <v>0</v>
       </c>
       <c r="E7" s="7" t="e">
@@ -911,28 +922,28 @@
         <v>0</v>
       </c>
       <c r="H7" s="9">
-        <v>1.5E-3</v>
+        <v>2E-3</v>
       </c>
       <c r="I7" s="6">
         <f>+G7*H7</f>
         <v>0</v>
       </c>
       <c r="L7" s="4"/>
-      <c r="M7" s="12"/>
+      <c r="M7" s="11"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C8" s="6">
-        <f>+SUMIFS('Perla del Mar'!L:L,'Perla del Mar'!P:P,Override!A8,'Perla del Mar'!F:F,"Comercial")</f>
+        <f>+SUMIFS('Carmelo Reservado'!L:L,'Carmelo Reservado'!P:P,Override!A8)</f>
         <v>0</v>
       </c>
       <c r="D8" s="6">
-        <f>+SUMIFS('Perla del Mar'!M:M,'Perla del Mar'!P:P,Override!A8,'Perla del Mar'!F:F,"Comercial")</f>
+        <f>+SUMIFS('Carmelo Reservado'!M:M,'Carmelo Reservado'!P:P,Override!A8)</f>
         <v>0</v>
       </c>
       <c r="E8" s="7" t="e">
@@ -940,7 +951,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="F8" s="6">
-        <f>+SUMIFS('Perla del Mar'!N:N,'Perla del Mar'!P:P,Override!A8,'Perla del Mar'!Q:Q,"No")</f>
+        <f>+SUMIFS('Carmelo Reservado'!N:N,'Carmelo Reservado'!P:P,Override!A8,'Carmelo Reservado'!Q:Q,"No")</f>
         <v>0</v>
       </c>
       <c r="G8" s="8">
@@ -948,519 +959,107 @@
         <v>0</v>
       </c>
       <c r="H8" s="9">
-        <v>1.5E-3</v>
+        <v>2E-3</v>
       </c>
       <c r="I8" s="6">
         <f>+G8*H8</f>
         <v>0</v>
       </c>
       <c r="L8" s="4"/>
-      <c r="M8" s="12"/>
+      <c r="M8" s="11"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="6">
-        <f>+SUMIFS('Carmelo Reservado'!L:L,'Carmelo Reservado'!P:P,Override!A9,'Carmelo Reservado'!F:F,"Comercial")</f>
+      <c r="A9" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="23"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="24"/>
+      <c r="I9" s="18">
+        <f>+I6+I7+I8</f>
         <v>0</v>
       </c>
-      <c r="D9" s="6">
-        <f>+SUMIFS('Carmelo Reservado'!M:M,'Carmelo Reservado'!P:P,Override!A9,'Carmelo Reservado'!F:F,"Comercial")</f>
-        <v>0</v>
-      </c>
-      <c r="E9" s="7" t="e">
-        <f>+D9/C9</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F9" s="6">
-        <f>+SUMIFS('Carmelo Reservado'!N:N,'Carmelo Reservado'!P:P,Override!A9,'Carmelo Reservado'!Q:Q,"No")</f>
-        <v>0</v>
-      </c>
-      <c r="G9" s="8">
-        <f>+D9+F9</f>
-        <v>0</v>
-      </c>
-      <c r="H9" s="9">
-        <v>1.5E-3</v>
-      </c>
-      <c r="I9" s="6">
-        <f>+G9*H9</f>
-        <v>0</v>
-      </c>
-      <c r="L9" s="4"/>
-      <c r="M9" s="12"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A10" s="20" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="10">
-        <f>SUM(I6:I9)</f>
-        <v>0</v>
-      </c>
-      <c r="L10" s="4"/>
-      <c r="M10" s="12"/>
-    </row>
-    <row r="11" spans="1:13" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="L11" s="4"/>
-      <c r="M11" s="12"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A12" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" s="6">
-        <f>+SUMIFS('Tesoro Escondido'!L:L,'Tesoro Escondido'!P:P,Override!A12,'Tesoro Escondido'!F:F,"Administrativa")</f>
-        <v>0</v>
-      </c>
-      <c r="D12" s="6">
-        <f>+SUMIFS('Tesoro Escondido'!M:M,'Tesoro Escondido'!P:P,Override!A12,'Tesoro Escondido'!F:F,"Administrativa")</f>
-        <v>0</v>
-      </c>
-      <c r="E12" s="7" t="e">
-        <f>+D12/C12</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F12" s="6">
-        <f>+SUMIFS('Tesoro Escondido'!N:N,'Tesoro Escondido'!P:P,Override!A12,'Tesoro Escondido'!Q:Q,"No")</f>
-        <v>0</v>
-      </c>
-      <c r="G12" s="8">
-        <f>+D12+F12</f>
-        <v>0</v>
-      </c>
-      <c r="H12" s="9">
-        <v>1.5E-3</v>
-      </c>
-      <c r="I12" s="6">
-        <f>+G12*H12</f>
-        <v>0</v>
-      </c>
-      <c r="L12" s="4"/>
-      <c r="M12" s="12"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A13" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" s="6">
-        <f>+SUMIFS('Vegas de Venecia'!L:L,'Vegas de Venecia'!P:P,Override!A13,'Vegas de Venecia'!F:F,"Administrativa")</f>
-        <v>0</v>
-      </c>
-      <c r="D13" s="6">
-        <f>+SUMIFS('Vegas de Venecia'!M:M,'Vegas de Venecia'!P:P,Override!A13,'Vegas de Venecia'!F:F,"Administrativa")</f>
-        <v>0</v>
-      </c>
-      <c r="E13" s="7" t="e">
-        <f>+D13/C13</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F13" s="6">
-        <f>+SUMIFS('Vegas de Venecia'!N:N,'Vegas de Venecia'!P:P,Override!A13,'Vegas de Venecia'!Q:Q,"No")</f>
-        <v>0</v>
-      </c>
-      <c r="G13" s="8">
-        <f>+D13+F13</f>
-        <v>0</v>
-      </c>
-      <c r="H13" s="9">
-        <v>1.5E-3</v>
-      </c>
-      <c r="I13" s="6">
-        <f>+G13*H13</f>
-        <v>0</v>
-      </c>
-      <c r="L13" s="4"/>
-      <c r="M13" s="12"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" s="6">
-        <f>+SUMIFS('Sandville Beach'!L:L,'Sandville Beach'!P:P,Override!A14,'Sandville Beach'!F:F,"Administrativa")</f>
-        <v>0</v>
-      </c>
-      <c r="D14" s="6">
-        <f>+SUMIFS('Sandville Beach'!M:M,'Sandville Beach'!P:P,Override!A14,'Sandville Beach'!F:F,"Administrativa")</f>
-        <v>0</v>
-      </c>
-      <c r="E14" s="7" t="e">
-        <f>+D14/C14</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F14" s="6">
-        <f>+SUMIFS('Sandville Beach'!N:N,'Sandville Beach'!P:P,Override!A14,'Sandville Beach'!Q:Q,"No")</f>
-        <v>0</v>
-      </c>
-      <c r="G14" s="8">
-        <f>+D14+F14</f>
-        <v>0</v>
-      </c>
-      <c r="H14" s="9">
-        <v>1.5E-3</v>
-      </c>
-      <c r="I14" s="6">
-        <f>+G14*H14</f>
-        <v>0</v>
-      </c>
-      <c r="L14" s="4"/>
-      <c r="M14" s="12"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" s="6">
-        <f>+SUMIFS('Carmelo Reservado'!L:L,'Carmelo Reservado'!P:P,Override!A15,'Carmelo Reservado'!F:F,"Administrativa")</f>
-        <v>0</v>
-      </c>
-      <c r="D15" s="6">
-        <f>+SUMIFS('Carmelo Reservado'!M:M,'Carmelo Reservado'!P:P,Override!A15,'Carmelo Reservado'!F:F,"Administrativa")</f>
-        <v>0</v>
-      </c>
-      <c r="E15" s="7" t="e">
-        <f>+D15/C15</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F15" s="6">
-        <f>+SUMIFS('Carmelo Reservado'!N:N,'Carmelo Reservado'!P:P,Override!A15,'Carmelo Reservado'!Q:Q,"No")</f>
-        <v>0</v>
-      </c>
-      <c r="G15" s="8">
-        <f>+D15+F15</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="9">
-        <v>1.5E-3</v>
-      </c>
-      <c r="I15" s="6">
-        <f>+G15*H15</f>
-        <v>0</v>
-      </c>
-      <c r="L15" s="4"/>
-      <c r="M15" s="12"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A16" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C16" s="6">
-        <f>+SUMIFS('Perla del Mar'!L:L,'Perla del Mar'!P:P,Override!A16,'Perla del Mar'!F:F,"Administrativa")</f>
-        <v>0</v>
-      </c>
-      <c r="D16" s="6">
-        <f>+SUMIFS('Perla del Mar'!M:M,'Perla del Mar'!P:P,Override!A16,'Perla del Mar'!F:F,"Administrativa")</f>
-        <v>0</v>
-      </c>
-      <c r="E16" s="7" t="e">
-        <f>+D16/C16</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F16" s="6">
-        <f>+SUMIFS('Perla del Mar'!N:N,'Perla del Mar'!P:P,Override!A16,'Perla del Mar'!Q:Q,"No")</f>
-        <v>0</v>
-      </c>
-      <c r="G16" s="8">
-        <f>+D16+F16</f>
-        <v>0</v>
-      </c>
-      <c r="H16" s="9">
-        <v>1.5E-3</v>
-      </c>
-      <c r="I16" s="6">
-        <f>+G16*H16</f>
-        <v>0</v>
-      </c>
-      <c r="L16" s="4"/>
-      <c r="M16" s="12"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A17" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
-      <c r="F17" s="21"/>
-      <c r="G17" s="21"/>
-      <c r="H17" s="22"/>
-      <c r="I17" s="10">
-        <f>SUM(I12:I16)</f>
-        <v>0</v>
-      </c>
-      <c r="L17" s="4"/>
-      <c r="M17" s="12"/>
-    </row>
-    <row r="18" spans="1:13" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C19" s="8">
-        <f>+C12</f>
-        <v>0</v>
-      </c>
-      <c r="D19" s="8">
-        <f>+D12</f>
-        <v>0</v>
-      </c>
-      <c r="E19" s="7" t="e">
-        <f>+D19/C19</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F19" s="8">
-        <f>+F12</f>
-        <v>0</v>
-      </c>
-      <c r="G19" s="8">
-        <f>+F19+D19</f>
-        <v>0</v>
-      </c>
-      <c r="H19" s="9" t="e">
-        <f>+IF(Override!E19&lt;Escalas!$A$3,Escalas!$B$2,IF(Override!E19&lt;Escalas!$A$4,Escalas!$B$3,IF(Override!E19&lt;Escalas!$A$5,Escalas!$B$4,Escalas!$B$5)))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I19" s="6" t="e">
-        <f>+G19*H19</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A20" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C20" s="8">
-        <f>+C13</f>
-        <v>0</v>
-      </c>
-      <c r="D20" s="8">
-        <f>+D13</f>
-        <v>0</v>
-      </c>
-      <c r="E20" s="7" t="e">
-        <f>+D20/C20</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F20" s="8">
-        <f>+F13</f>
-        <v>0</v>
-      </c>
-      <c r="G20" s="8">
-        <f>+F20+D20</f>
-        <v>0</v>
-      </c>
-      <c r="H20" s="9" t="e">
-        <f>+IF(Override!E20&lt;Escalas!$A$3,Escalas!$B$2,IF(Override!E20&lt;Escalas!$A$4,Escalas!$B$3,IF(Override!E20&lt;Escalas!$A$5,Escalas!$B$4,Escalas!$B$5)))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I20" s="6" t="e">
-        <f>+G20*H20</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C21" s="8">
-        <f>+C14+C2</f>
-        <v>0</v>
-      </c>
-      <c r="D21" s="8">
-        <f>+D14+D2</f>
-        <v>0</v>
-      </c>
-      <c r="E21" s="7" t="e">
-        <f>+D21/C21</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F21" s="8">
-        <f>+F14+F2</f>
-        <v>0</v>
-      </c>
-      <c r="G21" s="8">
-        <f>+F21+D21</f>
-        <v>0</v>
-      </c>
-      <c r="H21" s="9" t="e">
-        <f>+IF(Override!E21&lt;Escalas!$A$3,Escalas!$B$2,IF(Override!E21&lt;Escalas!$A$4,Escalas!$B$3,IF(Override!E21&lt;Escalas!$A$5,Escalas!$B$4,Escalas!$B$5)))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I21" s="6" t="e">
-        <f>+G21*H21</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A22" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C22" s="8">
-        <f>+C16+C3</f>
-        <v>0</v>
-      </c>
-      <c r="D22" s="8">
-        <f>+D16+D3</f>
-        <v>0</v>
-      </c>
-      <c r="E22" s="7" t="e">
-        <f>+D22/C22</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F22" s="8">
-        <f>+F16+F3+'Perla del Mar'!N37+'Perla del Mar'!N40</f>
-        <v>0</v>
-      </c>
-      <c r="G22" s="8">
-        <f>+F22+D22</f>
-        <v>0</v>
-      </c>
-      <c r="H22" s="9" t="e">
-        <f>+IF(Override!E22&lt;Escalas!$A$3,Escalas!$B$2,IF(Override!E22&lt;Escalas!$A$4,Escalas!$B$3,IF(Override!E22&lt;Escalas!$A$5,Escalas!$B$4,Escalas!$B$5)))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I22" s="6" t="e">
-        <f>+G22*H22</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A23" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="B23" s="21"/>
-      <c r="C23" s="21"/>
-      <c r="D23" s="21"/>
-      <c r="E23" s="21"/>
-      <c r="F23" s="21"/>
-      <c r="G23" s="21"/>
-      <c r="H23" s="22"/>
-      <c r="I23" s="10" t="e">
-        <f>SUM(I19:I22)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A24" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="B24" s="24"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="24"/>
-      <c r="H24" s="25"/>
-      <c r="I24" s="19" t="e">
-        <f>+I23+I17+I10</f>
-        <v>#DIV/0!</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A17:H17"/>
+  <mergeCells count="2">
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A9:H9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3BFFC70-E6BA-438E-9DBC-580D3A79AB7C}">
+  <dimension ref="A1:W1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="K1" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="L1" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="N1" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="O1" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="P1" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>35</v>
+      </c>
+      <c r="R1" s="14"/>
+      <c r="S1" s="14"/>
+      <c r="T1" s="14"/>
+      <c r="U1" s="14"/>
+      <c r="V1" s="14"/>
+      <c r="W1" s="14"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -1473,15 +1072,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" s="13" t="s">
-        <v>21</v>
+      <c r="A1" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="14">
+      <c r="A2" s="13">
         <v>0.4</v>
       </c>
       <c r="B2" s="9">
@@ -1489,7 +1088,7 @@
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="14">
+      <c r="A3" s="13">
         <v>0.6</v>
       </c>
       <c r="B3" s="9">
@@ -1497,7 +1096,7 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="14">
+      <c r="A4" s="13">
         <v>0.9</v>
       </c>
       <c r="B4" s="9">
@@ -1505,7 +1104,7 @@
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="14">
+      <c r="A5" s="13">
         <v>1</v>
       </c>
       <c r="B5" s="9">
@@ -1523,72 +1122,72 @@
   <dimension ref="A1:T16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.5546875" style="15" customWidth="1"/>
-    <col min="2" max="2" width="31.6640625" style="15" customWidth="1"/>
-    <col min="3" max="7" width="10.5546875" style="15" customWidth="1"/>
-    <col min="8" max="8" width="16" style="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.109375" style="15" customWidth="1"/>
-    <col min="10" max="10" width="21.21875" style="15" customWidth="1"/>
-    <col min="11" max="11" width="14.5546875" style="15" customWidth="1"/>
-    <col min="12" max="12" width="22.88671875" style="15" customWidth="1"/>
-    <col min="13" max="13" width="14.5546875" style="15" customWidth="1"/>
-    <col min="14" max="14" width="22.6640625" style="15" customWidth="1"/>
-    <col min="15" max="15" width="17.88671875" style="15" customWidth="1"/>
-    <col min="16" max="16" width="21.109375" style="15" customWidth="1"/>
-    <col min="17" max="20" width="10.5546875" style="15" customWidth="1"/>
+    <col min="1" max="1" width="10.5546875" style="14" customWidth="1"/>
+    <col min="2" max="2" width="31.6640625" style="14" customWidth="1"/>
+    <col min="3" max="7" width="10.5546875" style="14" customWidth="1"/>
+    <col min="8" max="8" width="16" style="14" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.109375" style="14" customWidth="1"/>
+    <col min="10" max="10" width="21.21875" style="14" customWidth="1"/>
+    <col min="11" max="11" width="14.5546875" style="14" customWidth="1"/>
+    <col min="12" max="12" width="22.88671875" style="14" customWidth="1"/>
+    <col min="13" max="13" width="14.5546875" style="14" customWidth="1"/>
+    <col min="14" max="14" width="22.6640625" style="14" customWidth="1"/>
+    <col min="15" max="15" width="17.88671875" style="14" customWidth="1"/>
+    <col min="16" max="16" width="21.109375" style="14" customWidth="1"/>
+    <col min="17" max="20" width="10.5546875" style="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
         <v>22</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
         <v>23</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
         <v>24</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" t="s">
         <v>25</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s">
         <v>26</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" t="s">
         <v>27</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" t="s">
         <v>28</v>
       </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
         <v>29</v>
       </c>
-      <c r="I1" t="s">
+      <c r="L1" t="s">
         <v>30</v>
       </c>
-      <c r="J1" t="s">
+      <c r="M1" t="s">
         <v>31</v>
       </c>
-      <c r="K1" t="s">
+      <c r="N1" t="s">
         <v>32</v>
       </c>
-      <c r="L1" t="s">
+      <c r="O1" t="s">
         <v>33</v>
       </c>
-      <c r="M1" t="s">
+      <c r="P1" t="s">
         <v>34</v>
       </c>
-      <c r="N1" t="s">
+      <c r="Q1" t="s">
         <v>35</v>
-      </c>
-      <c r="O1" t="s">
-        <v>36</v>
-      </c>
-      <c r="P1" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
@@ -1752,73 +1351,73 @@
   <dimension ref="A1:X110"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.5546875" style="15" customWidth="1"/>
-    <col min="2" max="2" width="44.21875" style="15" customWidth="1"/>
-    <col min="3" max="5" width="10.5546875" style="15" customWidth="1"/>
-    <col min="6" max="6" width="13.5546875" style="15" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" style="15" customWidth="1"/>
-    <col min="8" max="8" width="16.21875" style="15" customWidth="1"/>
-    <col min="9" max="9" width="19.109375" style="15" customWidth="1"/>
-    <col min="10" max="10" width="22.21875" style="15" customWidth="1"/>
-    <col min="11" max="12" width="23.33203125" style="15" customWidth="1"/>
-    <col min="13" max="13" width="18.5546875" style="15" customWidth="1"/>
-    <col min="14" max="14" width="25.21875" style="15" customWidth="1"/>
-    <col min="15" max="15" width="20" style="15" customWidth="1"/>
-    <col min="16" max="16" width="24.33203125" style="15" bestFit="1" customWidth="1"/>
-    <col min="17" max="24" width="10.5546875" style="15" customWidth="1"/>
+    <col min="1" max="1" width="10.5546875" style="14" customWidth="1"/>
+    <col min="2" max="2" width="44.21875" style="14" customWidth="1"/>
+    <col min="3" max="5" width="10.5546875" style="14" customWidth="1"/>
+    <col min="6" max="6" width="13.5546875" style="14" customWidth="1"/>
+    <col min="7" max="7" width="10.5546875" style="14" customWidth="1"/>
+    <col min="8" max="8" width="16.21875" style="14" customWidth="1"/>
+    <col min="9" max="9" width="19.109375" style="14" customWidth="1"/>
+    <col min="10" max="10" width="22.21875" style="14" customWidth="1"/>
+    <col min="11" max="12" width="23.33203125" style="14" customWidth="1"/>
+    <col min="13" max="13" width="18.5546875" style="14" customWidth="1"/>
+    <col min="14" max="14" width="25.21875" style="14" customWidth="1"/>
+    <col min="15" max="15" width="20" style="14" customWidth="1"/>
+    <col min="16" max="16" width="24.33203125" style="14" bestFit="1" customWidth="1"/>
+    <col min="17" max="24" width="10.5546875" style="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
         <v>22</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
         <v>23</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
         <v>24</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" t="s">
         <v>25</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s">
         <v>26</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" t="s">
         <v>27</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" t="s">
         <v>28</v>
       </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
         <v>29</v>
       </c>
-      <c r="I1" t="s">
+      <c r="L1" t="s">
         <v>30</v>
       </c>
-      <c r="J1" t="s">
+      <c r="M1" t="s">
         <v>31</v>
       </c>
-      <c r="K1" t="s">
+      <c r="N1" t="s">
         <v>32</v>
       </c>
-      <c r="L1" t="s">
+      <c r="O1" t="s">
         <v>33</v>
       </c>
-      <c r="M1" t="s">
+      <c r="P1" t="s">
         <v>34</v>
       </c>
-      <c r="N1" t="s">
+      <c r="Q1" t="s">
         <v>35</v>
-      </c>
-      <c r="O1" t="s">
-        <v>36</v>
-      </c>
-      <c r="P1" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
@@ -2922,76 +2521,76 @@
   <dimension ref="A1:V80"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.44140625" style="15" customWidth="1"/>
-    <col min="2" max="2" width="38.6640625" style="15" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" style="15" customWidth="1"/>
-    <col min="4" max="4" width="13.33203125" style="15" customWidth="1"/>
-    <col min="5" max="5" width="11.33203125" style="15" customWidth="1"/>
-    <col min="6" max="6" width="18" style="15" customWidth="1"/>
-    <col min="7" max="7" width="12.77734375" style="15" customWidth="1"/>
-    <col min="8" max="8" width="16.88671875" style="15" customWidth="1"/>
-    <col min="9" max="9" width="19.109375" style="15" customWidth="1"/>
-    <col min="10" max="10" width="22.21875" style="15" customWidth="1"/>
-    <col min="11" max="12" width="23.33203125" style="15" customWidth="1"/>
-    <col min="13" max="13" width="29.88671875" style="15" customWidth="1"/>
-    <col min="14" max="14" width="25.21875" style="15" customWidth="1"/>
-    <col min="15" max="15" width="20" style="15" customWidth="1"/>
-    <col min="16" max="16" width="22.21875" style="15" customWidth="1"/>
-    <col min="17" max="17" width="12.21875" style="15" customWidth="1"/>
-    <col min="18" max="22" width="8.88671875" style="15" customWidth="1"/>
+    <col min="1" max="1" width="15.44140625" style="14" customWidth="1"/>
+    <col min="2" max="2" width="38.6640625" style="14" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" style="14" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" style="14" customWidth="1"/>
+    <col min="5" max="5" width="11.33203125" style="14" customWidth="1"/>
+    <col min="6" max="6" width="18" style="14" customWidth="1"/>
+    <col min="7" max="7" width="12.77734375" style="14" customWidth="1"/>
+    <col min="8" max="8" width="16.88671875" style="14" customWidth="1"/>
+    <col min="9" max="9" width="19.109375" style="14" customWidth="1"/>
+    <col min="10" max="10" width="22.21875" style="14" customWidth="1"/>
+    <col min="11" max="12" width="23.33203125" style="14" customWidth="1"/>
+    <col min="13" max="13" width="29.88671875" style="14" customWidth="1"/>
+    <col min="14" max="14" width="25.21875" style="14" customWidth="1"/>
+    <col min="15" max="15" width="20" style="14" customWidth="1"/>
+    <col min="16" max="16" width="22.21875" style="14" customWidth="1"/>
+    <col min="17" max="17" width="12.21875" style="14" customWidth="1"/>
+    <col min="18" max="22" width="8.88671875" style="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
         <v>22</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
         <v>23</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
         <v>24</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" t="s">
         <v>25</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s">
         <v>26</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" t="s">
         <v>27</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" t="s">
         <v>28</v>
       </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
         <v>29</v>
       </c>
-      <c r="I1" t="s">
+      <c r="L1" t="s">
         <v>30</v>
       </c>
-      <c r="J1" t="s">
+      <c r="M1" t="s">
         <v>31</v>
       </c>
-      <c r="K1" t="s">
+      <c r="N1" t="s">
         <v>32</v>
       </c>
-      <c r="L1" t="s">
+      <c r="O1" t="s">
         <v>33</v>
       </c>
-      <c r="M1" t="s">
+      <c r="P1" t="s">
         <v>34</v>
       </c>
-      <c r="N1" t="s">
+      <c r="Q1" s="14" t="s">
         <v>35</v>
-      </c>
-      <c r="O1" t="s">
-        <v>36</v>
-      </c>
-      <c r="P1" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q1" s="15" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
@@ -3795,73 +3394,73 @@
   <dimension ref="A1:T38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.33203125" style="15" customWidth="1"/>
-    <col min="2" max="2" width="38.44140625" style="15" customWidth="1"/>
-    <col min="3" max="5" width="10.5546875" style="15" customWidth="1"/>
-    <col min="6" max="6" width="13.33203125" style="15" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" style="15" customWidth="1"/>
-    <col min="8" max="8" width="16.6640625" style="15" customWidth="1"/>
-    <col min="9" max="9" width="19.109375" style="15" customWidth="1"/>
-    <col min="10" max="10" width="22.21875" style="15" customWidth="1"/>
-    <col min="11" max="12" width="23.33203125" style="15" customWidth="1"/>
-    <col min="13" max="13" width="29.88671875" style="15" customWidth="1"/>
-    <col min="14" max="14" width="25.21875" style="15" customWidth="1"/>
-    <col min="15" max="15" width="20" style="15" customWidth="1"/>
-    <col min="16" max="16" width="24.33203125" style="15" customWidth="1"/>
-    <col min="17" max="20" width="10.5546875" style="15" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" style="14" customWidth="1"/>
+    <col min="2" max="2" width="38.44140625" style="14" customWidth="1"/>
+    <col min="3" max="5" width="10.5546875" style="14" customWidth="1"/>
+    <col min="6" max="6" width="13.33203125" style="14" customWidth="1"/>
+    <col min="7" max="7" width="10.5546875" style="14" customWidth="1"/>
+    <col min="8" max="8" width="16.6640625" style="14" customWidth="1"/>
+    <col min="9" max="9" width="19.109375" style="14" customWidth="1"/>
+    <col min="10" max="10" width="22.21875" style="14" customWidth="1"/>
+    <col min="11" max="12" width="23.33203125" style="14" customWidth="1"/>
+    <col min="13" max="13" width="29.88671875" style="14" customWidth="1"/>
+    <col min="14" max="14" width="25.21875" style="14" customWidth="1"/>
+    <col min="15" max="15" width="20" style="14" customWidth="1"/>
+    <col min="16" max="16" width="24.33203125" style="14" customWidth="1"/>
+    <col min="17" max="20" width="10.5546875" style="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
         <v>22</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
         <v>23</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
         <v>24</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" t="s">
         <v>25</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s">
         <v>26</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" t="s">
         <v>27</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" t="s">
         <v>28</v>
       </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
         <v>29</v>
       </c>
-      <c r="I1" t="s">
+      <c r="L1" t="s">
         <v>30</v>
       </c>
-      <c r="J1" t="s">
+      <c r="M1" t="s">
         <v>31</v>
       </c>
-      <c r="K1" t="s">
+      <c r="N1" t="s">
         <v>32</v>
       </c>
-      <c r="L1" t="s">
+      <c r="O1" t="s">
         <v>33</v>
       </c>
-      <c r="M1" t="s">
+      <c r="P1" t="s">
         <v>34</v>
       </c>
-      <c r="N1" t="s">
+      <c r="Q1" t="s">
         <v>35</v>
-      </c>
-      <c r="O1" t="s">
-        <v>36</v>
-      </c>
-      <c r="P1" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
@@ -4245,72 +3844,72 @@
   <dimension ref="A1:W111"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" style="15" customWidth="1"/>
-    <col min="2" max="2" width="41" style="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="7" width="11.5546875" style="15" customWidth="1"/>
-    <col min="8" max="8" width="14.6640625" style="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.88671875" style="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.88671875" style="15" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.88671875" style="15" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.88671875" style="15" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.88671875" style="15" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="24.109375" style="15" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.109375" style="15" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20" style="15" bestFit="1" customWidth="1"/>
-    <col min="17" max="23" width="11.5546875" style="15" customWidth="1"/>
+    <col min="1" max="1" width="11.5546875" style="14" customWidth="1"/>
+    <col min="2" max="2" width="41" style="14" bestFit="1" customWidth="1"/>
+    <col min="3" max="7" width="11.5546875" style="14" customWidth="1"/>
+    <col min="8" max="8" width="14.6640625" style="14" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.88671875" style="14" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.88671875" style="14" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.88671875" style="14" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.88671875" style="14" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.88671875" style="14" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="24.109375" style="14" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.109375" style="14" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20" style="14" bestFit="1" customWidth="1"/>
+    <col min="17" max="23" width="11.5546875" style="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
         <v>22</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
         <v>23</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
         <v>24</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" t="s">
         <v>25</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="K1" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="I1" s="15" t="s">
+      <c r="L1" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="J1" s="15" t="s">
+      <c r="M1" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="K1" s="15" t="s">
+      <c r="N1" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="L1" s="15" t="s">
+      <c r="O1" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="M1" s="15" t="s">
+      <c r="P1" t="s">
         <v>34</v>
       </c>
-      <c r="N1" s="15" t="s">
+      <c r="Q1" t="s">
         <v>35</v>
-      </c>
-      <c r="O1" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="P1" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
@@ -5423,255 +5022,255 @@
   <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="8" max="9" width="14.77734375" style="15" customWidth="1"/>
-    <col min="10" max="10" width="15.77734375" style="15" customWidth="1"/>
-    <col min="11" max="11" width="13.77734375" style="15" customWidth="1"/>
-    <col min="12" max="12" width="15.77734375" style="15" customWidth="1"/>
-    <col min="13" max="15" width="14.77734375" style="15" customWidth="1"/>
+    <col min="8" max="9" width="14.77734375" style="14" customWidth="1"/>
+    <col min="10" max="10" width="15.77734375" style="14" customWidth="1"/>
+    <col min="11" max="11" width="13.77734375" style="14" customWidth="1"/>
+    <col min="12" max="12" width="15.77734375" style="14" customWidth="1"/>
+    <col min="13" max="15" width="14.77734375" style="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
         <v>22</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
         <v>23</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
         <v>24</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" t="s">
         <v>25</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s">
         <v>26</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" t="s">
         <v>27</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" t="s">
         <v>28</v>
       </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
         <v>29</v>
       </c>
-      <c r="I1" t="s">
+      <c r="L1" t="s">
         <v>30</v>
       </c>
-      <c r="J1" t="s">
+      <c r="M1" t="s">
         <v>31</v>
       </c>
-      <c r="K1" t="s">
+      <c r="N1" t="s">
         <v>32</v>
       </c>
-      <c r="L1" t="s">
+      <c r="O1" t="s">
         <v>33</v>
       </c>
-      <c r="M1" t="s">
+      <c r="P1" t="s">
         <v>34</v>
       </c>
-      <c r="N1" t="s">
+      <c r="Q1" t="s">
         <v>35</v>
       </c>
-      <c r="O1" t="s">
-        <v>36</v>
-      </c>
-      <c r="P1" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>38</v>
-      </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A2" s="18"/>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="18"/>
-      <c r="M2" s="18"/>
-      <c r="N2" s="18"/>
-      <c r="O2" s="18"/>
-      <c r="P2" s="18"/>
+      <c r="A2" s="17"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="17"/>
+      <c r="M2" s="17"/>
+      <c r="N2" s="17"/>
+      <c r="O2" s="17"/>
+      <c r="P2" s="17"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A3" s="18"/>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
-      <c r="M3" s="18"/>
-      <c r="N3" s="18"/>
-      <c r="O3" s="18"/>
-      <c r="P3" s="18"/>
+      <c r="A3" s="17"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="17"/>
+      <c r="J3" s="17"/>
+      <c r="K3" s="17"/>
+      <c r="L3" s="17"/>
+      <c r="M3" s="17"/>
+      <c r="N3" s="17"/>
+      <c r="O3" s="17"/>
+      <c r="P3" s="17"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A4" s="17"/>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="L4" s="17"/>
-      <c r="M4" s="17"/>
-      <c r="N4" s="17"/>
-      <c r="O4" s="17"/>
-      <c r="P4" s="17"/>
+      <c r="A4" s="16"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="16"/>
+      <c r="J4" s="16"/>
+      <c r="K4" s="16"/>
+      <c r="L4" s="16"/>
+      <c r="M4" s="16"/>
+      <c r="N4" s="16"/>
+      <c r="O4" s="16"/>
+      <c r="P4" s="16"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A5" s="17"/>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="17"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="17"/>
-      <c r="M5" s="17"/>
-      <c r="N5" s="17"/>
-      <c r="O5" s="17"/>
-      <c r="P5" s="17"/>
+      <c r="A5" s="16"/>
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="16"/>
+      <c r="K5" s="16"/>
+      <c r="L5" s="16"/>
+      <c r="M5" s="16"/>
+      <c r="N5" s="16"/>
+      <c r="O5" s="16"/>
+      <c r="P5" s="16"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A6" s="17"/>
-      <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="17"/>
-      <c r="L6" s="17"/>
-      <c r="M6" s="17"/>
-      <c r="N6" s="17"/>
-      <c r="O6" s="17"/>
-      <c r="P6" s="17"/>
+      <c r="A6" s="16"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="16"/>
+      <c r="N6" s="16"/>
+      <c r="O6" s="16"/>
+      <c r="P6" s="16"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A7" s="17"/>
-      <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="17"/>
-      <c r="L7" s="17"/>
-      <c r="M7" s="17"/>
-      <c r="N7" s="17"/>
-      <c r="O7" s="17"/>
-      <c r="P7" s="17"/>
+      <c r="A7" s="16"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="16"/>
+      <c r="N7" s="16"/>
+      <c r="O7" s="16"/>
+      <c r="P7" s="16"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A8" s="17"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
-      <c r="L8" s="17"/>
-      <c r="M8" s="17"/>
-      <c r="N8" s="17"/>
-      <c r="O8" s="17"/>
-      <c r="P8" s="17"/>
+      <c r="A8" s="16"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="16"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="16"/>
+      <c r="N8" s="16"/>
+      <c r="O8" s="16"/>
+      <c r="P8" s="16"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A9" s="17"/>
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17"/>
-      <c r="M9" s="17"/>
-      <c r="N9" s="17"/>
-      <c r="O9" s="17"/>
-      <c r="P9" s="17"/>
+      <c r="A9" s="16"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="16"/>
+      <c r="L9" s="16"/>
+      <c r="M9" s="16"/>
+      <c r="N9" s="16"/>
+      <c r="O9" s="16"/>
+      <c r="P9" s="16"/>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A10" s="17"/>
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="17"/>
-      <c r="L10" s="17"/>
-      <c r="M10" s="17"/>
-      <c r="N10" s="17"/>
-      <c r="O10" s="17"/>
-      <c r="P10" s="17"/>
+      <c r="A10" s="16"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="16"/>
+      <c r="M10" s="16"/>
+      <c r="N10" s="16"/>
+      <c r="O10" s="16"/>
+      <c r="P10" s="16"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A11" s="17"/>
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
-      <c r="J11" s="17"/>
-      <c r="K11" s="17"/>
-      <c r="L11" s="17"/>
-      <c r="M11" s="17"/>
-      <c r="N11" s="17"/>
-      <c r="O11" s="17"/>
-      <c r="P11" s="17"/>
+      <c r="A11" s="16"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="16"/>
+      <c r="I11" s="16"/>
+      <c r="J11" s="16"/>
+      <c r="K11" s="16"/>
+      <c r="L11" s="16"/>
+      <c r="M11" s="16"/>
+      <c r="N11" s="16"/>
+      <c r="O11" s="16"/>
+      <c r="P11" s="16"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A12" s="16"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="P12" s="16"/>
+      <c r="A12" s="15"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="P12" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -5680,68 +5279,68 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3BFFC70-E6BA-438E-9DBC-580D3A79AB7C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8768682F-933C-494D-9284-3785B686D543}">
   <dimension ref="A1:W1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
         <v>22</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
         <v>23</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
         <v>24</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" t="s">
         <v>25</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="K1" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="I1" s="15" t="s">
+      <c r="L1" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="J1" s="15" t="s">
+      <c r="M1" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="K1" s="15" t="s">
+      <c r="N1" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="L1" s="15" t="s">
+      <c r="O1" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="M1" s="15" t="s">
+      <c r="P1" t="s">
         <v>34</v>
       </c>
-      <c r="N1" s="15" t="s">
+      <c r="Q1" t="s">
         <v>35</v>
       </c>
-      <c r="O1" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="P1" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>38</v>
-      </c>
-      <c r="R1" s="15"/>
-      <c r="S1" s="15"/>
-      <c r="T1" s="15"/>
-      <c r="U1" s="15"/>
-      <c r="V1" s="15"/>
-      <c r="W1" s="15"/>
+      <c r="R1" s="14"/>
+      <c r="S1" s="14"/>
+      <c r="T1" s="14"/>
+      <c r="U1" s="14"/>
+      <c r="V1" s="14"/>
+      <c r="W1" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>